<commit_message>
fix(routing): add client-side dynamic route fallback and auto-load Explore data
</commit_message>
<xml_diff>
--- a/TripSync_TestReport.xlsx
+++ b/TripSync_TestReport.xlsx
@@ -552,7 +552,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>23.11 seconds</t>
+          <t>37.28 seconds</t>
         </is>
       </c>
     </row>
@@ -6000,7 +6000,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>1.326</v>
+        <v>2.189</v>
       </c>
       <c r="F2" t="inlineStr"/>
     </row>
@@ -6026,7 +6026,7 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>0.22</v>
+        <v>0.321</v>
       </c>
       <c r="F3" t="inlineStr"/>
     </row>
@@ -6052,7 +6052,7 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>0.22</v>
+        <v>0.631</v>
       </c>
       <c r="F4" t="inlineStr"/>
     </row>
@@ -6078,7 +6078,7 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>0.253</v>
+        <v>0.382</v>
       </c>
       <c r="F5" t="inlineStr"/>
     </row>
@@ -6104,7 +6104,7 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>0.218</v>
+        <v>0.267</v>
       </c>
       <c r="F6" t="inlineStr"/>
     </row>
@@ -6130,7 +6130,7 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>0.221</v>
+        <v>0.346</v>
       </c>
       <c r="F7" t="inlineStr"/>
     </row>
@@ -6156,7 +6156,7 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>0.222</v>
+        <v>0.447</v>
       </c>
       <c r="F8" t="inlineStr"/>
     </row>
@@ -6182,7 +6182,7 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>0.217</v>
+        <v>0.297</v>
       </c>
       <c r="F9" t="inlineStr"/>
     </row>
@@ -6208,7 +6208,7 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>0.218</v>
+        <v>0.331</v>
       </c>
       <c r="F10" t="inlineStr"/>
     </row>
@@ -6234,7 +6234,7 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>0.216</v>
+        <v>0.355</v>
       </c>
       <c r="F11" t="inlineStr"/>
     </row>
@@ -6260,7 +6260,7 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>0.217</v>
+        <v>0.248</v>
       </c>
       <c r="F12" t="inlineStr"/>
     </row>
@@ -6286,7 +6286,7 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>0.218</v>
+        <v>0.349</v>
       </c>
       <c r="F13" t="inlineStr"/>
     </row>
@@ -6312,7 +6312,7 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>0.218</v>
+        <v>0.235</v>
       </c>
       <c r="F14" t="inlineStr"/>
     </row>
@@ -6338,7 +6338,7 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>0.22</v>
+        <v>0.283</v>
       </c>
       <c r="F15" t="inlineStr"/>
     </row>
@@ -6364,7 +6364,7 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>0.22</v>
+        <v>0.343</v>
       </c>
       <c r="F16" t="inlineStr"/>
     </row>
@@ -6390,7 +6390,7 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>0.22</v>
+        <v>0.369</v>
       </c>
       <c r="F17" t="inlineStr"/>
     </row>
@@ -6416,7 +6416,7 @@
         </is>
       </c>
       <c r="E18" t="n">
-        <v>0.249</v>
+        <v>0.355</v>
       </c>
       <c r="F18" t="inlineStr"/>
     </row>
@@ -6442,7 +6442,7 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>0.217</v>
+        <v>0.386</v>
       </c>
       <c r="F19" t="inlineStr"/>
     </row>
@@ -6468,7 +6468,7 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>0.217</v>
+        <v>0.427</v>
       </c>
       <c r="F20" t="inlineStr"/>
     </row>
@@ -6494,7 +6494,7 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>0.217</v>
+        <v>0.28</v>
       </c>
       <c r="F21" t="inlineStr"/>
     </row>
@@ -6520,7 +6520,7 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>0.216</v>
+        <v>0.58</v>
       </c>
       <c r="F22" t="inlineStr"/>
     </row>
@@ -6546,7 +6546,7 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>0.216</v>
+        <v>0.307</v>
       </c>
       <c r="F23" t="inlineStr"/>
     </row>
@@ -6572,7 +6572,7 @@
         </is>
       </c>
       <c r="E24" t="n">
-        <v>0.217</v>
+        <v>0.311</v>
       </c>
       <c r="F24" t="inlineStr"/>
     </row>
@@ -6598,7 +6598,7 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>0.222</v>
+        <v>0.296</v>
       </c>
       <c r="F25" t="inlineStr"/>
     </row>
@@ -6624,7 +6624,7 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>0.217</v>
+        <v>0.246</v>
       </c>
       <c r="F26" t="inlineStr"/>
     </row>
@@ -6650,7 +6650,7 @@
         </is>
       </c>
       <c r="E27" t="n">
-        <v>0.22</v>
+        <v>0.54</v>
       </c>
       <c r="F27" t="inlineStr"/>
     </row>
@@ -6676,7 +6676,7 @@
         </is>
       </c>
       <c r="E28" t="n">
-        <v>0.216</v>
+        <v>0.346</v>
       </c>
       <c r="F28" t="inlineStr"/>
     </row>
@@ -6702,7 +6702,7 @@
         </is>
       </c>
       <c r="E29" t="n">
-        <v>0.217</v>
+        <v>0.548</v>
       </c>
       <c r="F29" t="inlineStr"/>
     </row>
@@ -6728,7 +6728,7 @@
         </is>
       </c>
       <c r="E30" t="n">
-        <v>0.218</v>
+        <v>0.967</v>
       </c>
       <c r="F30" t="inlineStr"/>
     </row>
@@ -6754,7 +6754,7 @@
         </is>
       </c>
       <c r="E31" t="n">
-        <v>0.256</v>
+        <v>0.281</v>
       </c>
       <c r="F31" t="inlineStr"/>
     </row>
@@ -6780,7 +6780,7 @@
         </is>
       </c>
       <c r="E32" t="n">
-        <v>0.219</v>
+        <v>0.403</v>
       </c>
       <c r="F32" t="inlineStr"/>
     </row>
@@ -6806,7 +6806,7 @@
         </is>
       </c>
       <c r="E33" t="n">
-        <v>0.217</v>
+        <v>0.294</v>
       </c>
       <c r="F33" t="inlineStr"/>
     </row>
@@ -6832,7 +6832,7 @@
         </is>
       </c>
       <c r="E34" t="n">
-        <v>0.216</v>
+        <v>0.249</v>
       </c>
       <c r="F34" t="inlineStr"/>
     </row>
@@ -6858,7 +6858,7 @@
         </is>
       </c>
       <c r="E35" t="n">
-        <v>0.224</v>
+        <v>0.338</v>
       </c>
       <c r="F35" t="inlineStr"/>
     </row>
@@ -6884,7 +6884,7 @@
         </is>
       </c>
       <c r="E36" t="n">
-        <v>0.219</v>
+        <v>0.238</v>
       </c>
       <c r="F36" t="inlineStr"/>
     </row>
@@ -6910,7 +6910,7 @@
         </is>
       </c>
       <c r="E37" t="n">
-        <v>0.216</v>
+        <v>0.305</v>
       </c>
       <c r="F37" t="inlineStr"/>
     </row>
@@ -6936,7 +6936,7 @@
         </is>
       </c>
       <c r="E38" t="n">
-        <v>0.219</v>
+        <v>0.725</v>
       </c>
       <c r="F38" t="inlineStr"/>
     </row>
@@ -6962,7 +6962,7 @@
         </is>
       </c>
       <c r="E39" t="n">
-        <v>0.218</v>
+        <v>0.319</v>
       </c>
       <c r="F39" t="inlineStr"/>
     </row>
@@ -6988,7 +6988,7 @@
         </is>
       </c>
       <c r="E40" t="n">
-        <v>0.219</v>
+        <v>0.426</v>
       </c>
       <c r="F40" t="inlineStr"/>
     </row>
@@ -7014,7 +7014,7 @@
         </is>
       </c>
       <c r="E41" t="n">
-        <v>0.219</v>
+        <v>0.252</v>
       </c>
       <c r="F41" t="inlineStr"/>
     </row>
@@ -7040,7 +7040,7 @@
         </is>
       </c>
       <c r="E42" t="n">
-        <v>0.226</v>
+        <v>0.543</v>
       </c>
       <c r="F42" t="inlineStr"/>
     </row>
@@ -7066,7 +7066,7 @@
         </is>
       </c>
       <c r="E43" t="n">
-        <v>0.252</v>
+        <v>0.234</v>
       </c>
       <c r="F43" t="inlineStr"/>
     </row>
@@ -7092,7 +7092,7 @@
         </is>
       </c>
       <c r="E44" t="n">
-        <v>0.217</v>
+        <v>0.326</v>
       </c>
       <c r="F44" t="inlineStr"/>
     </row>
@@ -7118,7 +7118,7 @@
         </is>
       </c>
       <c r="E45" t="n">
-        <v>0.218</v>
+        <v>0.248</v>
       </c>
       <c r="F45" t="inlineStr"/>
     </row>
@@ -7144,7 +7144,7 @@
         </is>
       </c>
       <c r="E46" t="n">
-        <v>0.218</v>
+        <v>0.239</v>
       </c>
       <c r="F46" t="inlineStr"/>
     </row>
@@ -7170,7 +7170,7 @@
         </is>
       </c>
       <c r="E47" t="n">
-        <v>0.216</v>
+        <v>0.898</v>
       </c>
       <c r="F47" t="inlineStr"/>
     </row>
@@ -7196,7 +7196,7 @@
         </is>
       </c>
       <c r="E48" t="n">
-        <v>0.217</v>
+        <v>0.246</v>
       </c>
       <c r="F48" t="inlineStr"/>
     </row>
@@ -7222,7 +7222,7 @@
         </is>
       </c>
       <c r="E49" t="n">
-        <v>0.223</v>
+        <v>0.374</v>
       </c>
       <c r="F49" t="inlineStr"/>
     </row>
@@ -7248,7 +7248,7 @@
         </is>
       </c>
       <c r="E50" t="n">
-        <v>0.217</v>
+        <v>0.303</v>
       </c>
       <c r="F50" t="inlineStr"/>
     </row>
@@ -7274,7 +7274,7 @@
         </is>
       </c>
       <c r="E51" t="n">
-        <v>0.217</v>
+        <v>0.239</v>
       </c>
       <c r="F51" t="inlineStr"/>
     </row>
@@ -7300,7 +7300,7 @@
         </is>
       </c>
       <c r="E52" t="n">
-        <v>0.214</v>
+        <v>0.263</v>
       </c>
       <c r="F52" t="inlineStr"/>
     </row>
@@ -7326,7 +7326,7 @@
         </is>
       </c>
       <c r="E53" t="n">
-        <v>0.217</v>
+        <v>0.29</v>
       </c>
       <c r="F53" t="inlineStr"/>
     </row>
@@ -7352,7 +7352,7 @@
         </is>
       </c>
       <c r="E54" t="n">
-        <v>0.217</v>
+        <v>0.247</v>
       </c>
       <c r="F54" t="inlineStr"/>
     </row>
@@ -7378,7 +7378,7 @@
         </is>
       </c>
       <c r="E55" t="n">
-        <v>0.219</v>
+        <v>0.294</v>
       </c>
       <c r="F55" t="inlineStr"/>
     </row>
@@ -7404,7 +7404,7 @@
         </is>
       </c>
       <c r="E56" t="n">
-        <v>0.254</v>
+        <v>0.246</v>
       </c>
       <c r="F56" t="inlineStr"/>
     </row>
@@ -7430,7 +7430,7 @@
         </is>
       </c>
       <c r="E57" t="n">
-        <v>0.216</v>
+        <v>0.263</v>
       </c>
       <c r="F57" t="inlineStr"/>
     </row>
@@ -7456,7 +7456,7 @@
         </is>
       </c>
       <c r="E58" t="n">
-        <v>0.219</v>
+        <v>0.407</v>
       </c>
       <c r="F58" t="inlineStr"/>
     </row>
@@ -7482,7 +7482,7 @@
         </is>
       </c>
       <c r="E59" t="n">
-        <v>0.216</v>
+        <v>0.245</v>
       </c>
       <c r="F59" t="inlineStr"/>
     </row>
@@ -7508,7 +7508,7 @@
         </is>
       </c>
       <c r="E60" t="n">
-        <v>0.218</v>
+        <v>0.266</v>
       </c>
       <c r="F60" t="inlineStr"/>
     </row>
@@ -7534,7 +7534,7 @@
         </is>
       </c>
       <c r="E61" t="n">
-        <v>0.217</v>
+        <v>0.62</v>
       </c>
       <c r="F61" t="inlineStr"/>
     </row>
@@ -7560,7 +7560,7 @@
         </is>
       </c>
       <c r="E62" t="n">
-        <v>0.218</v>
+        <v>0.293</v>
       </c>
       <c r="F62" t="inlineStr"/>
     </row>
@@ -7586,7 +7586,7 @@
         </is>
       </c>
       <c r="E63" t="n">
-        <v>0.218</v>
+        <v>0.871</v>
       </c>
       <c r="F63" t="inlineStr"/>
     </row>
@@ -7612,7 +7612,7 @@
         </is>
       </c>
       <c r="E64" t="n">
-        <v>0.217</v>
+        <v>0.509</v>
       </c>
       <c r="F64" t="inlineStr"/>
     </row>
@@ -7638,7 +7638,7 @@
         </is>
       </c>
       <c r="E65" t="n">
-        <v>0.219</v>
+        <v>0.245</v>
       </c>
       <c r="F65" t="inlineStr"/>
     </row>
@@ -7664,7 +7664,7 @@
         </is>
       </c>
       <c r="E66" t="n">
-        <v>0.219</v>
+        <v>0.315</v>
       </c>
       <c r="F66" t="inlineStr"/>
     </row>
@@ -7690,7 +7690,7 @@
         </is>
       </c>
       <c r="E67" t="n">
-        <v>0.217</v>
+        <v>0.337</v>
       </c>
       <c r="F67" t="inlineStr"/>
     </row>
@@ -7716,7 +7716,7 @@
         </is>
       </c>
       <c r="E68" t="n">
-        <v>0.218</v>
+        <v>0.334</v>
       </c>
       <c r="F68" t="inlineStr"/>
     </row>
@@ -7742,7 +7742,7 @@
         </is>
       </c>
       <c r="E69" t="n">
-        <v>0.216</v>
+        <v>0.496</v>
       </c>
       <c r="F69" t="inlineStr"/>
     </row>
@@ -7768,7 +7768,7 @@
         </is>
       </c>
       <c r="E70" t="n">
-        <v>0.218</v>
+        <v>0.255</v>
       </c>
       <c r="F70" t="inlineStr"/>
     </row>
@@ -7794,7 +7794,7 @@
         </is>
       </c>
       <c r="E71" t="n">
-        <v>0.217</v>
+        <v>0.389</v>
       </c>
       <c r="F71" t="inlineStr"/>
     </row>
@@ -7820,7 +7820,7 @@
         </is>
       </c>
       <c r="E72" t="n">
-        <v>0.22</v>
+        <v>0.224</v>
       </c>
       <c r="F72" t="inlineStr"/>
     </row>
@@ -7846,7 +7846,7 @@
         </is>
       </c>
       <c r="E73" t="n">
-        <v>0.218</v>
+        <v>0.232</v>
       </c>
       <c r="F73" t="inlineStr"/>
     </row>
@@ -7872,7 +7872,7 @@
         </is>
       </c>
       <c r="E74" t="n">
-        <v>0.222</v>
+        <v>0.34</v>
       </c>
       <c r="F74" t="inlineStr"/>
     </row>
@@ -7898,7 +7898,7 @@
         </is>
       </c>
       <c r="E75" t="n">
-        <v>0.218</v>
+        <v>0.276</v>
       </c>
       <c r="F75" t="inlineStr"/>
     </row>
@@ -7924,7 +7924,7 @@
         </is>
       </c>
       <c r="E76" t="n">
-        <v>0.218</v>
+        <v>0.703</v>
       </c>
       <c r="F76" t="inlineStr"/>
     </row>
@@ -7950,7 +7950,7 @@
         </is>
       </c>
       <c r="E77" t="n">
-        <v>0.219</v>
+        <v>0.37</v>
       </c>
       <c r="F77" t="inlineStr"/>
     </row>
@@ -7976,7 +7976,7 @@
         </is>
       </c>
       <c r="E78" t="n">
-        <v>0.216</v>
+        <v>0.259</v>
       </c>
       <c r="F78" t="inlineStr"/>
     </row>
@@ -8002,7 +8002,7 @@
         </is>
       </c>
       <c r="E79" t="n">
-        <v>0.219</v>
+        <v>0.242</v>
       </c>
       <c r="F79" t="inlineStr"/>
     </row>
@@ -8028,7 +8028,7 @@
         </is>
       </c>
       <c r="E80" t="n">
-        <v>0.217</v>
+        <v>0.251</v>
       </c>
       <c r="F80" t="inlineStr"/>
     </row>
@@ -8054,7 +8054,7 @@
         </is>
       </c>
       <c r="E81" t="n">
-        <v>0.218</v>
+        <v>0.281</v>
       </c>
       <c r="F81" t="inlineStr"/>
     </row>
@@ -8080,7 +8080,7 @@
         </is>
       </c>
       <c r="E82" t="n">
-        <v>0.217</v>
+        <v>0.31</v>
       </c>
       <c r="F82" t="inlineStr"/>
     </row>
@@ -8106,7 +8106,7 @@
         </is>
       </c>
       <c r="E83" t="n">
-        <v>0.222</v>
+        <v>0.26</v>
       </c>
       <c r="F83" t="inlineStr"/>
     </row>
@@ -8132,7 +8132,7 @@
         </is>
       </c>
       <c r="E84" t="n">
-        <v>0.217</v>
+        <v>0.26</v>
       </c>
       <c r="F84" t="inlineStr"/>
     </row>
@@ -8158,7 +8158,7 @@
         </is>
       </c>
       <c r="E85" t="n">
-        <v>0.218</v>
+        <v>0.265</v>
       </c>
       <c r="F85" t="inlineStr"/>
     </row>
@@ -8184,7 +8184,7 @@
         </is>
       </c>
       <c r="E86" t="n">
-        <v>0.22</v>
+        <v>0.306</v>
       </c>
       <c r="F86" t="inlineStr"/>
     </row>
@@ -8210,7 +8210,7 @@
         </is>
       </c>
       <c r="E87" t="n">
-        <v>0.217</v>
+        <v>0.328</v>
       </c>
       <c r="F87" t="inlineStr"/>
     </row>
@@ -8236,7 +8236,7 @@
         </is>
       </c>
       <c r="E88" t="n">
-        <v>0.219</v>
+        <v>0.468</v>
       </c>
       <c r="F88" t="inlineStr"/>
     </row>
@@ -8262,7 +8262,7 @@
         </is>
       </c>
       <c r="E89" t="n">
-        <v>0.215</v>
+        <v>0.27</v>
       </c>
       <c r="F89" t="inlineStr"/>
     </row>
@@ -8288,7 +8288,7 @@
         </is>
       </c>
       <c r="E90" t="n">
-        <v>0.216</v>
+        <v>0.241</v>
       </c>
       <c r="F90" t="inlineStr"/>
     </row>
@@ -8314,7 +8314,7 @@
         </is>
       </c>
       <c r="E91" t="n">
-        <v>0.217</v>
+        <v>0.306</v>
       </c>
       <c r="F91" t="inlineStr"/>
     </row>
@@ -8340,7 +8340,7 @@
         </is>
       </c>
       <c r="E92" t="n">
-        <v>0.217</v>
+        <v>0.336</v>
       </c>
       <c r="F92" t="inlineStr"/>
     </row>
@@ -8366,7 +8366,7 @@
         </is>
       </c>
       <c r="E93" t="n">
-        <v>0.218</v>
+        <v>0.235</v>
       </c>
       <c r="F93" t="inlineStr"/>
     </row>
@@ -8392,7 +8392,7 @@
         </is>
       </c>
       <c r="E94" t="n">
-        <v>0.218</v>
+        <v>0.419</v>
       </c>
       <c r="F94" t="inlineStr"/>
     </row>
@@ -8418,7 +8418,7 @@
         </is>
       </c>
       <c r="E95" t="n">
-        <v>0.216</v>
+        <v>0.574</v>
       </c>
       <c r="F95" t="inlineStr"/>
     </row>
@@ -8444,7 +8444,7 @@
         </is>
       </c>
       <c r="E96" t="n">
-        <v>0.216</v>
+        <v>0.29</v>
       </c>
       <c r="F96" t="inlineStr"/>
     </row>
@@ -8470,7 +8470,7 @@
         </is>
       </c>
       <c r="E97" t="n">
-        <v>0.218</v>
+        <v>0.271</v>
       </c>
       <c r="F97" t="inlineStr"/>
     </row>
@@ -8496,7 +8496,7 @@
         </is>
       </c>
       <c r="E98" t="n">
-        <v>0.217</v>
+        <v>0.306</v>
       </c>
       <c r="F98" t="inlineStr"/>
     </row>
@@ -8522,7 +8522,7 @@
         </is>
       </c>
       <c r="E99" t="n">
-        <v>0.215</v>
+        <v>0.363</v>
       </c>
       <c r="F99" t="inlineStr"/>
     </row>
@@ -8548,7 +8548,7 @@
         </is>
       </c>
       <c r="E100" t="n">
-        <v>0.218</v>
+        <v>0.358</v>
       </c>
       <c r="F100" t="inlineStr"/>
     </row>
@@ -8574,7 +8574,7 @@
         </is>
       </c>
       <c r="E101" t="n">
-        <v>0.216</v>
+        <v>0.263</v>
       </c>
       <c r="F101" t="inlineStr"/>
     </row>
@@ -13938,7 +13938,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>1.326</v>
+        <v>2.189</v>
       </c>
       <c r="F2" t="inlineStr"/>
     </row>
@@ -13964,7 +13964,7 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>0.22</v>
+        <v>0.321</v>
       </c>
       <c r="F3" t="inlineStr"/>
     </row>
@@ -13990,7 +13990,7 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>0.22</v>
+        <v>0.631</v>
       </c>
       <c r="F4" t="inlineStr"/>
     </row>
@@ -14016,7 +14016,7 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>0.253</v>
+        <v>0.382</v>
       </c>
       <c r="F5" t="inlineStr"/>
     </row>
@@ -14042,7 +14042,7 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>0.218</v>
+        <v>0.267</v>
       </c>
       <c r="F6" t="inlineStr"/>
     </row>
@@ -14068,7 +14068,7 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>0.221</v>
+        <v>0.346</v>
       </c>
       <c r="F7" t="inlineStr"/>
     </row>
@@ -14094,7 +14094,7 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>0.222</v>
+        <v>0.447</v>
       </c>
       <c r="F8" t="inlineStr"/>
     </row>
@@ -14120,7 +14120,7 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>0.217</v>
+        <v>0.297</v>
       </c>
       <c r="F9" t="inlineStr"/>
     </row>
@@ -14146,7 +14146,7 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>0.218</v>
+        <v>0.331</v>
       </c>
       <c r="F10" t="inlineStr"/>
     </row>
@@ -14172,7 +14172,7 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>0.216</v>
+        <v>0.355</v>
       </c>
       <c r="F11" t="inlineStr"/>
     </row>
@@ -14198,7 +14198,7 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>0.217</v>
+        <v>0.248</v>
       </c>
       <c r="F12" t="inlineStr"/>
     </row>
@@ -14224,7 +14224,7 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>0.218</v>
+        <v>0.349</v>
       </c>
       <c r="F13" t="inlineStr"/>
     </row>
@@ -14250,7 +14250,7 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>0.218</v>
+        <v>0.235</v>
       </c>
       <c r="F14" t="inlineStr"/>
     </row>
@@ -14276,7 +14276,7 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>0.22</v>
+        <v>0.283</v>
       </c>
       <c r="F15" t="inlineStr"/>
     </row>
@@ -14302,7 +14302,7 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>0.22</v>
+        <v>0.343</v>
       </c>
       <c r="F16" t="inlineStr"/>
     </row>
@@ -14328,7 +14328,7 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>0.22</v>
+        <v>0.369</v>
       </c>
       <c r="F17" t="inlineStr"/>
     </row>
@@ -14354,7 +14354,7 @@
         </is>
       </c>
       <c r="E18" t="n">
-        <v>0.249</v>
+        <v>0.355</v>
       </c>
       <c r="F18" t="inlineStr"/>
     </row>
@@ -14380,7 +14380,7 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>0.217</v>
+        <v>0.386</v>
       </c>
       <c r="F19" t="inlineStr"/>
     </row>
@@ -14406,7 +14406,7 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>0.217</v>
+        <v>0.427</v>
       </c>
       <c r="F20" t="inlineStr"/>
     </row>
@@ -14432,7 +14432,7 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>0.217</v>
+        <v>0.28</v>
       </c>
       <c r="F21" t="inlineStr"/>
     </row>
@@ -14458,7 +14458,7 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>0.216</v>
+        <v>0.58</v>
       </c>
       <c r="F22" t="inlineStr"/>
     </row>
@@ -14484,7 +14484,7 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>0.216</v>
+        <v>0.307</v>
       </c>
       <c r="F23" t="inlineStr"/>
     </row>
@@ -14510,7 +14510,7 @@
         </is>
       </c>
       <c r="E24" t="n">
-        <v>0.217</v>
+        <v>0.311</v>
       </c>
       <c r="F24" t="inlineStr"/>
     </row>
@@ -14536,7 +14536,7 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>0.222</v>
+        <v>0.296</v>
       </c>
       <c r="F25" t="inlineStr"/>
     </row>
@@ -14562,7 +14562,7 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>0.217</v>
+        <v>0.246</v>
       </c>
       <c r="F26" t="inlineStr"/>
     </row>
@@ -14588,7 +14588,7 @@
         </is>
       </c>
       <c r="E27" t="n">
-        <v>0.22</v>
+        <v>0.54</v>
       </c>
       <c r="F27" t="inlineStr"/>
     </row>
@@ -14614,7 +14614,7 @@
         </is>
       </c>
       <c r="E28" t="n">
-        <v>0.216</v>
+        <v>0.346</v>
       </c>
       <c r="F28" t="inlineStr"/>
     </row>
@@ -14640,7 +14640,7 @@
         </is>
       </c>
       <c r="E29" t="n">
-        <v>0.217</v>
+        <v>0.548</v>
       </c>
       <c r="F29" t="inlineStr"/>
     </row>
@@ -14666,7 +14666,7 @@
         </is>
       </c>
       <c r="E30" t="n">
-        <v>0.218</v>
+        <v>0.967</v>
       </c>
       <c r="F30" t="inlineStr"/>
     </row>
@@ -14692,7 +14692,7 @@
         </is>
       </c>
       <c r="E31" t="n">
-        <v>0.256</v>
+        <v>0.281</v>
       </c>
       <c r="F31" t="inlineStr"/>
     </row>
@@ -14718,7 +14718,7 @@
         </is>
       </c>
       <c r="E32" t="n">
-        <v>0.219</v>
+        <v>0.403</v>
       </c>
       <c r="F32" t="inlineStr"/>
     </row>
@@ -14744,7 +14744,7 @@
         </is>
       </c>
       <c r="E33" t="n">
-        <v>0.217</v>
+        <v>0.294</v>
       </c>
       <c r="F33" t="inlineStr"/>
     </row>
@@ -14770,7 +14770,7 @@
         </is>
       </c>
       <c r="E34" t="n">
-        <v>0.216</v>
+        <v>0.249</v>
       </c>
       <c r="F34" t="inlineStr"/>
     </row>
@@ -14796,7 +14796,7 @@
         </is>
       </c>
       <c r="E35" t="n">
-        <v>0.224</v>
+        <v>0.338</v>
       </c>
       <c r="F35" t="inlineStr"/>
     </row>
@@ -14822,7 +14822,7 @@
         </is>
       </c>
       <c r="E36" t="n">
-        <v>0.219</v>
+        <v>0.238</v>
       </c>
       <c r="F36" t="inlineStr"/>
     </row>
@@ -14848,7 +14848,7 @@
         </is>
       </c>
       <c r="E37" t="n">
-        <v>0.216</v>
+        <v>0.305</v>
       </c>
       <c r="F37" t="inlineStr"/>
     </row>
@@ -14874,7 +14874,7 @@
         </is>
       </c>
       <c r="E38" t="n">
-        <v>0.219</v>
+        <v>0.725</v>
       </c>
       <c r="F38" t="inlineStr"/>
     </row>
@@ -14900,7 +14900,7 @@
         </is>
       </c>
       <c r="E39" t="n">
-        <v>0.218</v>
+        <v>0.319</v>
       </c>
       <c r="F39" t="inlineStr"/>
     </row>
@@ -14926,7 +14926,7 @@
         </is>
       </c>
       <c r="E40" t="n">
-        <v>0.219</v>
+        <v>0.426</v>
       </c>
       <c r="F40" t="inlineStr"/>
     </row>
@@ -14952,7 +14952,7 @@
         </is>
       </c>
       <c r="E41" t="n">
-        <v>0.219</v>
+        <v>0.252</v>
       </c>
       <c r="F41" t="inlineStr"/>
     </row>
@@ -14978,7 +14978,7 @@
         </is>
       </c>
       <c r="E42" t="n">
-        <v>0.226</v>
+        <v>0.543</v>
       </c>
       <c r="F42" t="inlineStr"/>
     </row>
@@ -15004,7 +15004,7 @@
         </is>
       </c>
       <c r="E43" t="n">
-        <v>0.252</v>
+        <v>0.234</v>
       </c>
       <c r="F43" t="inlineStr"/>
     </row>
@@ -15030,7 +15030,7 @@
         </is>
       </c>
       <c r="E44" t="n">
-        <v>0.217</v>
+        <v>0.326</v>
       </c>
       <c r="F44" t="inlineStr"/>
     </row>
@@ -15056,7 +15056,7 @@
         </is>
       </c>
       <c r="E45" t="n">
-        <v>0.218</v>
+        <v>0.248</v>
       </c>
       <c r="F45" t="inlineStr"/>
     </row>
@@ -15082,7 +15082,7 @@
         </is>
       </c>
       <c r="E46" t="n">
-        <v>0.218</v>
+        <v>0.239</v>
       </c>
       <c r="F46" t="inlineStr"/>
     </row>
@@ -15108,7 +15108,7 @@
         </is>
       </c>
       <c r="E47" t="n">
-        <v>0.216</v>
+        <v>0.898</v>
       </c>
       <c r="F47" t="inlineStr"/>
     </row>
@@ -15134,7 +15134,7 @@
         </is>
       </c>
       <c r="E48" t="n">
-        <v>0.217</v>
+        <v>0.246</v>
       </c>
       <c r="F48" t="inlineStr"/>
     </row>
@@ -15160,7 +15160,7 @@
         </is>
       </c>
       <c r="E49" t="n">
-        <v>0.223</v>
+        <v>0.374</v>
       </c>
       <c r="F49" t="inlineStr"/>
     </row>
@@ -15186,7 +15186,7 @@
         </is>
       </c>
       <c r="E50" t="n">
-        <v>0.217</v>
+        <v>0.303</v>
       </c>
       <c r="F50" t="inlineStr"/>
     </row>
@@ -15212,7 +15212,7 @@
         </is>
       </c>
       <c r="E51" t="n">
-        <v>0.217</v>
+        <v>0.239</v>
       </c>
       <c r="F51" t="inlineStr"/>
     </row>
@@ -15238,7 +15238,7 @@
         </is>
       </c>
       <c r="E52" t="n">
-        <v>0.214</v>
+        <v>0.263</v>
       </c>
       <c r="F52" t="inlineStr"/>
     </row>
@@ -15264,7 +15264,7 @@
         </is>
       </c>
       <c r="E53" t="n">
-        <v>0.217</v>
+        <v>0.29</v>
       </c>
       <c r="F53" t="inlineStr"/>
     </row>
@@ -15290,7 +15290,7 @@
         </is>
       </c>
       <c r="E54" t="n">
-        <v>0.217</v>
+        <v>0.247</v>
       </c>
       <c r="F54" t="inlineStr"/>
     </row>
@@ -15316,7 +15316,7 @@
         </is>
       </c>
       <c r="E55" t="n">
-        <v>0.219</v>
+        <v>0.294</v>
       </c>
       <c r="F55" t="inlineStr"/>
     </row>
@@ -15342,7 +15342,7 @@
         </is>
       </c>
       <c r="E56" t="n">
-        <v>0.254</v>
+        <v>0.246</v>
       </c>
       <c r="F56" t="inlineStr"/>
     </row>
@@ -15368,7 +15368,7 @@
         </is>
       </c>
       <c r="E57" t="n">
-        <v>0.216</v>
+        <v>0.263</v>
       </c>
       <c r="F57" t="inlineStr"/>
     </row>
@@ -15394,7 +15394,7 @@
         </is>
       </c>
       <c r="E58" t="n">
-        <v>0.219</v>
+        <v>0.407</v>
       </c>
       <c r="F58" t="inlineStr"/>
     </row>
@@ -15420,7 +15420,7 @@
         </is>
       </c>
       <c r="E59" t="n">
-        <v>0.216</v>
+        <v>0.245</v>
       </c>
       <c r="F59" t="inlineStr"/>
     </row>
@@ -15446,7 +15446,7 @@
         </is>
       </c>
       <c r="E60" t="n">
-        <v>0.218</v>
+        <v>0.266</v>
       </c>
       <c r="F60" t="inlineStr"/>
     </row>
@@ -15472,7 +15472,7 @@
         </is>
       </c>
       <c r="E61" t="n">
-        <v>0.217</v>
+        <v>0.62</v>
       </c>
       <c r="F61" t="inlineStr"/>
     </row>
@@ -15498,7 +15498,7 @@
         </is>
       </c>
       <c r="E62" t="n">
-        <v>0.218</v>
+        <v>0.293</v>
       </c>
       <c r="F62" t="inlineStr"/>
     </row>
@@ -15524,7 +15524,7 @@
         </is>
       </c>
       <c r="E63" t="n">
-        <v>0.218</v>
+        <v>0.871</v>
       </c>
       <c r="F63" t="inlineStr"/>
     </row>
@@ -15550,7 +15550,7 @@
         </is>
       </c>
       <c r="E64" t="n">
-        <v>0.217</v>
+        <v>0.509</v>
       </c>
       <c r="F64" t="inlineStr"/>
     </row>
@@ -15576,7 +15576,7 @@
         </is>
       </c>
       <c r="E65" t="n">
-        <v>0.219</v>
+        <v>0.245</v>
       </c>
       <c r="F65" t="inlineStr"/>
     </row>
@@ -15602,7 +15602,7 @@
         </is>
       </c>
       <c r="E66" t="n">
-        <v>0.219</v>
+        <v>0.315</v>
       </c>
       <c r="F66" t="inlineStr"/>
     </row>
@@ -15628,7 +15628,7 @@
         </is>
       </c>
       <c r="E67" t="n">
-        <v>0.217</v>
+        <v>0.337</v>
       </c>
       <c r="F67" t="inlineStr"/>
     </row>
@@ -15654,7 +15654,7 @@
         </is>
       </c>
       <c r="E68" t="n">
-        <v>0.218</v>
+        <v>0.334</v>
       </c>
       <c r="F68" t="inlineStr"/>
     </row>
@@ -15680,7 +15680,7 @@
         </is>
       </c>
       <c r="E69" t="n">
-        <v>0.216</v>
+        <v>0.496</v>
       </c>
       <c r="F69" t="inlineStr"/>
     </row>
@@ -15706,7 +15706,7 @@
         </is>
       </c>
       <c r="E70" t="n">
-        <v>0.218</v>
+        <v>0.255</v>
       </c>
       <c r="F70" t="inlineStr"/>
     </row>
@@ -15732,7 +15732,7 @@
         </is>
       </c>
       <c r="E71" t="n">
-        <v>0.217</v>
+        <v>0.389</v>
       </c>
       <c r="F71" t="inlineStr"/>
     </row>
@@ -15758,7 +15758,7 @@
         </is>
       </c>
       <c r="E72" t="n">
-        <v>0.22</v>
+        <v>0.224</v>
       </c>
       <c r="F72" t="inlineStr"/>
     </row>
@@ -15784,7 +15784,7 @@
         </is>
       </c>
       <c r="E73" t="n">
-        <v>0.218</v>
+        <v>0.232</v>
       </c>
       <c r="F73" t="inlineStr"/>
     </row>
@@ -15810,7 +15810,7 @@
         </is>
       </c>
       <c r="E74" t="n">
-        <v>0.222</v>
+        <v>0.34</v>
       </c>
       <c r="F74" t="inlineStr"/>
     </row>
@@ -15836,7 +15836,7 @@
         </is>
       </c>
       <c r="E75" t="n">
-        <v>0.218</v>
+        <v>0.276</v>
       </c>
       <c r="F75" t="inlineStr"/>
     </row>
@@ -15862,7 +15862,7 @@
         </is>
       </c>
       <c r="E76" t="n">
-        <v>0.218</v>
+        <v>0.703</v>
       </c>
       <c r="F76" t="inlineStr"/>
     </row>
@@ -15888,7 +15888,7 @@
         </is>
       </c>
       <c r="E77" t="n">
-        <v>0.219</v>
+        <v>0.37</v>
       </c>
       <c r="F77" t="inlineStr"/>
     </row>
@@ -15914,7 +15914,7 @@
         </is>
       </c>
       <c r="E78" t="n">
-        <v>0.216</v>
+        <v>0.259</v>
       </c>
       <c r="F78" t="inlineStr"/>
     </row>
@@ -15940,7 +15940,7 @@
         </is>
       </c>
       <c r="E79" t="n">
-        <v>0.219</v>
+        <v>0.242</v>
       </c>
       <c r="F79" t="inlineStr"/>
     </row>
@@ -15966,7 +15966,7 @@
         </is>
       </c>
       <c r="E80" t="n">
-        <v>0.217</v>
+        <v>0.251</v>
       </c>
       <c r="F80" t="inlineStr"/>
     </row>
@@ -15992,7 +15992,7 @@
         </is>
       </c>
       <c r="E81" t="n">
-        <v>0.218</v>
+        <v>0.281</v>
       </c>
       <c r="F81" t="inlineStr"/>
     </row>
@@ -16018,7 +16018,7 @@
         </is>
       </c>
       <c r="E82" t="n">
-        <v>0.217</v>
+        <v>0.31</v>
       </c>
       <c r="F82" t="inlineStr"/>
     </row>
@@ -16044,7 +16044,7 @@
         </is>
       </c>
       <c r="E83" t="n">
-        <v>0.222</v>
+        <v>0.26</v>
       </c>
       <c r="F83" t="inlineStr"/>
     </row>
@@ -16070,7 +16070,7 @@
         </is>
       </c>
       <c r="E84" t="n">
-        <v>0.217</v>
+        <v>0.26</v>
       </c>
       <c r="F84" t="inlineStr"/>
     </row>
@@ -16096,7 +16096,7 @@
         </is>
       </c>
       <c r="E85" t="n">
-        <v>0.218</v>
+        <v>0.265</v>
       </c>
       <c r="F85" t="inlineStr"/>
     </row>
@@ -16122,7 +16122,7 @@
         </is>
       </c>
       <c r="E86" t="n">
-        <v>0.22</v>
+        <v>0.306</v>
       </c>
       <c r="F86" t="inlineStr"/>
     </row>
@@ -16148,7 +16148,7 @@
         </is>
       </c>
       <c r="E87" t="n">
-        <v>0.217</v>
+        <v>0.328</v>
       </c>
       <c r="F87" t="inlineStr"/>
     </row>
@@ -16174,7 +16174,7 @@
         </is>
       </c>
       <c r="E88" t="n">
-        <v>0.219</v>
+        <v>0.468</v>
       </c>
       <c r="F88" t="inlineStr"/>
     </row>
@@ -16200,7 +16200,7 @@
         </is>
       </c>
       <c r="E89" t="n">
-        <v>0.215</v>
+        <v>0.27</v>
       </c>
       <c r="F89" t="inlineStr"/>
     </row>
@@ -16226,7 +16226,7 @@
         </is>
       </c>
       <c r="E90" t="n">
-        <v>0.216</v>
+        <v>0.241</v>
       </c>
       <c r="F90" t="inlineStr"/>
     </row>
@@ -16252,7 +16252,7 @@
         </is>
       </c>
       <c r="E91" t="n">
-        <v>0.217</v>
+        <v>0.306</v>
       </c>
       <c r="F91" t="inlineStr"/>
     </row>
@@ -16278,7 +16278,7 @@
         </is>
       </c>
       <c r="E92" t="n">
-        <v>0.217</v>
+        <v>0.336</v>
       </c>
       <c r="F92" t="inlineStr"/>
     </row>
@@ -16304,7 +16304,7 @@
         </is>
       </c>
       <c r="E93" t="n">
-        <v>0.218</v>
+        <v>0.235</v>
       </c>
       <c r="F93" t="inlineStr"/>
     </row>
@@ -16330,7 +16330,7 @@
         </is>
       </c>
       <c r="E94" t="n">
-        <v>0.218</v>
+        <v>0.419</v>
       </c>
       <c r="F94" t="inlineStr"/>
     </row>
@@ -16356,7 +16356,7 @@
         </is>
       </c>
       <c r="E95" t="n">
-        <v>0.216</v>
+        <v>0.574</v>
       </c>
       <c r="F95" t="inlineStr"/>
     </row>
@@ -16382,7 +16382,7 @@
         </is>
       </c>
       <c r="E96" t="n">
-        <v>0.216</v>
+        <v>0.29</v>
       </c>
       <c r="F96" t="inlineStr"/>
     </row>
@@ -16408,7 +16408,7 @@
         </is>
       </c>
       <c r="E97" t="n">
-        <v>0.218</v>
+        <v>0.271</v>
       </c>
       <c r="F97" t="inlineStr"/>
     </row>
@@ -16434,7 +16434,7 @@
         </is>
       </c>
       <c r="E98" t="n">
-        <v>0.217</v>
+        <v>0.306</v>
       </c>
       <c r="F98" t="inlineStr"/>
     </row>
@@ -16460,7 +16460,7 @@
         </is>
       </c>
       <c r="E99" t="n">
-        <v>0.215</v>
+        <v>0.363</v>
       </c>
       <c r="F99" t="inlineStr"/>
     </row>
@@ -16486,7 +16486,7 @@
         </is>
       </c>
       <c r="E100" t="n">
-        <v>0.218</v>
+        <v>0.358</v>
       </c>
       <c r="F100" t="inlineStr"/>
     </row>
@@ -16512,7 +16512,7 @@
         </is>
       </c>
       <c r="E101" t="n">
-        <v>0.216</v>
+        <v>0.263</v>
       </c>
       <c r="F101" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
fix(expenses): add 5s storage timeout, finally block, and Base64 fallback to prevent infinite receipt upload spinner
</commit_message>
<xml_diff>
--- a/TripSync_TestReport.xlsx
+++ b/TripSync_TestReport.xlsx
@@ -463,7 +463,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>767</v>
+        <v>760</v>
       </c>
     </row>
     <row r="5">
@@ -552,7 +552,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>37.28 seconds</t>
+          <t>66.43 seconds</t>
         </is>
       </c>
     </row>
@@ -6000,7 +6000,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>2.189</v>
+        <v>4.234</v>
       </c>
       <c r="F2" t="inlineStr"/>
     </row>
@@ -6026,7 +6026,7 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>0.321</v>
+        <v>3.317</v>
       </c>
       <c r="F3" t="inlineStr"/>
     </row>
@@ -6052,7 +6052,7 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>0.631</v>
+        <v>3.336</v>
       </c>
       <c r="F4" t="inlineStr"/>
     </row>
@@ -6078,7 +6078,7 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>0.382</v>
+        <v>3.285</v>
       </c>
       <c r="F5" t="inlineStr"/>
     </row>
@@ -6104,7 +6104,7 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>0.267</v>
+        <v>3.343</v>
       </c>
       <c r="F6" t="inlineStr"/>
     </row>
@@ -6130,7 +6130,7 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>0.346</v>
+        <v>3.224</v>
       </c>
       <c r="F7" t="inlineStr"/>
     </row>
@@ -6156,7 +6156,7 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>0.447</v>
+        <v>3.267</v>
       </c>
       <c r="F8" t="inlineStr"/>
     </row>
@@ -6182,7 +6182,7 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>0.297</v>
+        <v>1.597</v>
       </c>
       <c r="F9" t="inlineStr"/>
     </row>
@@ -6208,7 +6208,7 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>0.331</v>
+        <v>0.891</v>
       </c>
       <c r="F10" t="inlineStr"/>
     </row>
@@ -6234,7 +6234,7 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>0.355</v>
+        <v>0.984</v>
       </c>
       <c r="F11" t="inlineStr"/>
     </row>
@@ -6260,7 +6260,7 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>0.248</v>
+        <v>0.224</v>
       </c>
       <c r="F12" t="inlineStr"/>
     </row>
@@ -6286,7 +6286,7 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>0.349</v>
+        <v>0.351</v>
       </c>
       <c r="F13" t="inlineStr"/>
     </row>
@@ -6312,7 +6312,7 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>0.235</v>
+        <v>0.223</v>
       </c>
       <c r="F14" t="inlineStr"/>
     </row>
@@ -6338,7 +6338,7 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>0.283</v>
+        <v>0.254</v>
       </c>
       <c r="F15" t="inlineStr"/>
     </row>
@@ -6364,7 +6364,7 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>0.343</v>
+        <v>0.281</v>
       </c>
       <c r="F16" t="inlineStr"/>
     </row>
@@ -6390,7 +6390,7 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>0.369</v>
+        <v>0.219</v>
       </c>
       <c r="F17" t="inlineStr"/>
     </row>
@@ -6416,7 +6416,7 @@
         </is>
       </c>
       <c r="E18" t="n">
-        <v>0.355</v>
+        <v>0.232</v>
       </c>
       <c r="F18" t="inlineStr"/>
     </row>
@@ -6442,7 +6442,7 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>0.386</v>
+        <v>0.285</v>
       </c>
       <c r="F19" t="inlineStr"/>
     </row>
@@ -6468,7 +6468,7 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>0.427</v>
+        <v>0.217</v>
       </c>
       <c r="F20" t="inlineStr"/>
     </row>
@@ -6494,7 +6494,7 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>0.28</v>
+        <v>0.242</v>
       </c>
       <c r="F21" t="inlineStr"/>
     </row>
@@ -6520,7 +6520,7 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>0.58</v>
+        <v>0.284</v>
       </c>
       <c r="F22" t="inlineStr"/>
     </row>
@@ -6546,7 +6546,7 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>0.307</v>
+        <v>0.226</v>
       </c>
       <c r="F23" t="inlineStr"/>
     </row>
@@ -6572,7 +6572,7 @@
         </is>
       </c>
       <c r="E24" t="n">
-        <v>0.311</v>
+        <v>0.238</v>
       </c>
       <c r="F24" t="inlineStr"/>
     </row>
@@ -6598,7 +6598,7 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>0.296</v>
+        <v>0.223</v>
       </c>
       <c r="F25" t="inlineStr"/>
     </row>
@@ -6624,7 +6624,7 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>0.246</v>
+        <v>0.235</v>
       </c>
       <c r="F26" t="inlineStr"/>
     </row>
@@ -6650,7 +6650,7 @@
         </is>
       </c>
       <c r="E27" t="n">
-        <v>0.54</v>
+        <v>0.225</v>
       </c>
       <c r="F27" t="inlineStr"/>
     </row>
@@ -6676,7 +6676,7 @@
         </is>
       </c>
       <c r="E28" t="n">
-        <v>0.346</v>
+        <v>0.249</v>
       </c>
       <c r="F28" t="inlineStr"/>
     </row>
@@ -6702,7 +6702,7 @@
         </is>
       </c>
       <c r="E29" t="n">
-        <v>0.548</v>
+        <v>0.296</v>
       </c>
       <c r="F29" t="inlineStr"/>
     </row>
@@ -6728,7 +6728,7 @@
         </is>
       </c>
       <c r="E30" t="n">
-        <v>0.967</v>
+        <v>0.222</v>
       </c>
       <c r="F30" t="inlineStr"/>
     </row>
@@ -6754,7 +6754,7 @@
         </is>
       </c>
       <c r="E31" t="n">
-        <v>0.281</v>
+        <v>0.223</v>
       </c>
       <c r="F31" t="inlineStr"/>
     </row>
@@ -6780,7 +6780,7 @@
         </is>
       </c>
       <c r="E32" t="n">
-        <v>0.403</v>
+        <v>0.375</v>
       </c>
       <c r="F32" t="inlineStr"/>
     </row>
@@ -6806,7 +6806,7 @@
         </is>
       </c>
       <c r="E33" t="n">
-        <v>0.294</v>
+        <v>0.246</v>
       </c>
       <c r="F33" t="inlineStr"/>
     </row>
@@ -6832,7 +6832,7 @@
         </is>
       </c>
       <c r="E34" t="n">
-        <v>0.249</v>
+        <v>0.252</v>
       </c>
       <c r="F34" t="inlineStr"/>
     </row>
@@ -6858,7 +6858,7 @@
         </is>
       </c>
       <c r="E35" t="n">
-        <v>0.338</v>
+        <v>0.255</v>
       </c>
       <c r="F35" t="inlineStr"/>
     </row>
@@ -6884,7 +6884,7 @@
         </is>
       </c>
       <c r="E36" t="n">
-        <v>0.238</v>
+        <v>0.302</v>
       </c>
       <c r="F36" t="inlineStr"/>
     </row>
@@ -6910,7 +6910,7 @@
         </is>
       </c>
       <c r="E37" t="n">
-        <v>0.305</v>
+        <v>0.246</v>
       </c>
       <c r="F37" t="inlineStr"/>
     </row>
@@ -6936,7 +6936,7 @@
         </is>
       </c>
       <c r="E38" t="n">
-        <v>0.725</v>
+        <v>0.231</v>
       </c>
       <c r="F38" t="inlineStr"/>
     </row>
@@ -6962,7 +6962,7 @@
         </is>
       </c>
       <c r="E39" t="n">
-        <v>0.319</v>
+        <v>0.22</v>
       </c>
       <c r="F39" t="inlineStr"/>
     </row>
@@ -6988,7 +6988,7 @@
         </is>
       </c>
       <c r="E40" t="n">
-        <v>0.426</v>
+        <v>0.407</v>
       </c>
       <c r="F40" t="inlineStr"/>
     </row>
@@ -7014,7 +7014,7 @@
         </is>
       </c>
       <c r="E41" t="n">
-        <v>0.252</v>
+        <v>0.222</v>
       </c>
       <c r="F41" t="inlineStr"/>
     </row>
@@ -7040,7 +7040,7 @@
         </is>
       </c>
       <c r="E42" t="n">
-        <v>0.543</v>
+        <v>0.832</v>
       </c>
       <c r="F42" t="inlineStr"/>
     </row>
@@ -7092,7 +7092,7 @@
         </is>
       </c>
       <c r="E44" t="n">
-        <v>0.326</v>
+        <v>0.443</v>
       </c>
       <c r="F44" t="inlineStr"/>
     </row>
@@ -7118,7 +7118,7 @@
         </is>
       </c>
       <c r="E45" t="n">
-        <v>0.248</v>
+        <v>0.29</v>
       </c>
       <c r="F45" t="inlineStr"/>
     </row>
@@ -7144,7 +7144,7 @@
         </is>
       </c>
       <c r="E46" t="n">
-        <v>0.239</v>
+        <v>0.227</v>
       </c>
       <c r="F46" t="inlineStr"/>
     </row>
@@ -7170,7 +7170,7 @@
         </is>
       </c>
       <c r="E47" t="n">
-        <v>0.898</v>
+        <v>0.219</v>
       </c>
       <c r="F47" t="inlineStr"/>
     </row>
@@ -7196,7 +7196,7 @@
         </is>
       </c>
       <c r="E48" t="n">
-        <v>0.246</v>
+        <v>0.758</v>
       </c>
       <c r="F48" t="inlineStr"/>
     </row>
@@ -7222,7 +7222,7 @@
         </is>
       </c>
       <c r="E49" t="n">
-        <v>0.374</v>
+        <v>0.261</v>
       </c>
       <c r="F49" t="inlineStr"/>
     </row>
@@ -7248,7 +7248,7 @@
         </is>
       </c>
       <c r="E50" t="n">
-        <v>0.303</v>
+        <v>0.219</v>
       </c>
       <c r="F50" t="inlineStr"/>
     </row>
@@ -7274,7 +7274,7 @@
         </is>
       </c>
       <c r="E51" t="n">
-        <v>0.239</v>
+        <v>0.22</v>
       </c>
       <c r="F51" t="inlineStr"/>
     </row>
@@ -7300,7 +7300,7 @@
         </is>
       </c>
       <c r="E52" t="n">
-        <v>0.263</v>
+        <v>0.22</v>
       </c>
       <c r="F52" t="inlineStr"/>
     </row>
@@ -7326,7 +7326,7 @@
         </is>
       </c>
       <c r="E53" t="n">
-        <v>0.29</v>
+        <v>0.252</v>
       </c>
       <c r="F53" t="inlineStr"/>
     </row>
@@ -7352,7 +7352,7 @@
         </is>
       </c>
       <c r="E54" t="n">
-        <v>0.247</v>
+        <v>0.262</v>
       </c>
       <c r="F54" t="inlineStr"/>
     </row>
@@ -7378,7 +7378,7 @@
         </is>
       </c>
       <c r="E55" t="n">
-        <v>0.294</v>
+        <v>2.016</v>
       </c>
       <c r="F55" t="inlineStr"/>
     </row>
@@ -7404,7 +7404,7 @@
         </is>
       </c>
       <c r="E56" t="n">
-        <v>0.246</v>
+        <v>4.025</v>
       </c>
       <c r="F56" t="inlineStr"/>
     </row>
@@ -7430,7 +7430,7 @@
         </is>
       </c>
       <c r="E57" t="n">
-        <v>0.263</v>
+        <v>2.127</v>
       </c>
       <c r="F57" t="inlineStr"/>
     </row>
@@ -7456,7 +7456,7 @@
         </is>
       </c>
       <c r="E58" t="n">
-        <v>0.407</v>
+        <v>1.194</v>
       </c>
       <c r="F58" t="inlineStr"/>
     </row>
@@ -7482,7 +7482,7 @@
         </is>
       </c>
       <c r="E59" t="n">
-        <v>0.245</v>
+        <v>0.575</v>
       </c>
       <c r="F59" t="inlineStr"/>
     </row>
@@ -7508,7 +7508,7 @@
         </is>
       </c>
       <c r="E60" t="n">
-        <v>0.266</v>
+        <v>0.286</v>
       </c>
       <c r="F60" t="inlineStr"/>
     </row>
@@ -7534,7 +7534,7 @@
         </is>
       </c>
       <c r="E61" t="n">
-        <v>0.62</v>
+        <v>0.283</v>
       </c>
       <c r="F61" t="inlineStr"/>
     </row>
@@ -7560,7 +7560,7 @@
         </is>
       </c>
       <c r="E62" t="n">
-        <v>0.293</v>
+        <v>0.337</v>
       </c>
       <c r="F62" t="inlineStr"/>
     </row>
@@ -7586,7 +7586,7 @@
         </is>
       </c>
       <c r="E63" t="n">
-        <v>0.871</v>
+        <v>0.283</v>
       </c>
       <c r="F63" t="inlineStr"/>
     </row>
@@ -7612,7 +7612,7 @@
         </is>
       </c>
       <c r="E64" t="n">
-        <v>0.509</v>
+        <v>0.241</v>
       </c>
       <c r="F64" t="inlineStr"/>
     </row>
@@ -7638,7 +7638,7 @@
         </is>
       </c>
       <c r="E65" t="n">
-        <v>0.245</v>
+        <v>0.414</v>
       </c>
       <c r="F65" t="inlineStr"/>
     </row>
@@ -7664,7 +7664,7 @@
         </is>
       </c>
       <c r="E66" t="n">
-        <v>0.315</v>
+        <v>0.477</v>
       </c>
       <c r="F66" t="inlineStr"/>
     </row>
@@ -7690,7 +7690,7 @@
         </is>
       </c>
       <c r="E67" t="n">
-        <v>0.337</v>
+        <v>0.24</v>
       </c>
       <c r="F67" t="inlineStr"/>
     </row>
@@ -7716,7 +7716,7 @@
         </is>
       </c>
       <c r="E68" t="n">
-        <v>0.334</v>
+        <v>0.297</v>
       </c>
       <c r="F68" t="inlineStr"/>
     </row>
@@ -7742,7 +7742,7 @@
         </is>
       </c>
       <c r="E69" t="n">
-        <v>0.496</v>
+        <v>0.308</v>
       </c>
       <c r="F69" t="inlineStr"/>
     </row>
@@ -7768,7 +7768,7 @@
         </is>
       </c>
       <c r="E70" t="n">
-        <v>0.255</v>
+        <v>0.236</v>
       </c>
       <c r="F70" t="inlineStr"/>
     </row>
@@ -7794,7 +7794,7 @@
         </is>
       </c>
       <c r="E71" t="n">
-        <v>0.389</v>
+        <v>0.24</v>
       </c>
       <c r="F71" t="inlineStr"/>
     </row>
@@ -7820,7 +7820,7 @@
         </is>
       </c>
       <c r="E72" t="n">
-        <v>0.224</v>
+        <v>0.269</v>
       </c>
       <c r="F72" t="inlineStr"/>
     </row>
@@ -7846,7 +7846,7 @@
         </is>
       </c>
       <c r="E73" t="n">
-        <v>0.232</v>
+        <v>0.274</v>
       </c>
       <c r="F73" t="inlineStr"/>
     </row>
@@ -7872,7 +7872,7 @@
         </is>
       </c>
       <c r="E74" t="n">
-        <v>0.34</v>
+        <v>0.24</v>
       </c>
       <c r="F74" t="inlineStr"/>
     </row>
@@ -7898,7 +7898,7 @@
         </is>
       </c>
       <c r="E75" t="n">
-        <v>0.276</v>
+        <v>0.641</v>
       </c>
       <c r="F75" t="inlineStr"/>
     </row>
@@ -7924,7 +7924,7 @@
         </is>
       </c>
       <c r="E76" t="n">
-        <v>0.703</v>
+        <v>0.611</v>
       </c>
       <c r="F76" t="inlineStr"/>
     </row>
@@ -7950,7 +7950,7 @@
         </is>
       </c>
       <c r="E77" t="n">
-        <v>0.37</v>
+        <v>0.25</v>
       </c>
       <c r="F77" t="inlineStr"/>
     </row>
@@ -7976,7 +7976,7 @@
         </is>
       </c>
       <c r="E78" t="n">
-        <v>0.259</v>
+        <v>0.342</v>
       </c>
       <c r="F78" t="inlineStr"/>
     </row>
@@ -8002,7 +8002,7 @@
         </is>
       </c>
       <c r="E79" t="n">
-        <v>0.242</v>
+        <v>0.771</v>
       </c>
       <c r="F79" t="inlineStr"/>
     </row>
@@ -8028,7 +8028,7 @@
         </is>
       </c>
       <c r="E80" t="n">
-        <v>0.251</v>
+        <v>0.599</v>
       </c>
       <c r="F80" t="inlineStr"/>
     </row>
@@ -8054,7 +8054,7 @@
         </is>
       </c>
       <c r="E81" t="n">
-        <v>0.281</v>
+        <v>0.488</v>
       </c>
       <c r="F81" t="inlineStr"/>
     </row>
@@ -8080,7 +8080,7 @@
         </is>
       </c>
       <c r="E82" t="n">
-        <v>0.31</v>
+        <v>0.244</v>
       </c>
       <c r="F82" t="inlineStr"/>
     </row>
@@ -8106,7 +8106,7 @@
         </is>
       </c>
       <c r="E83" t="n">
-        <v>0.26</v>
+        <v>0.575</v>
       </c>
       <c r="F83" t="inlineStr"/>
     </row>
@@ -8132,7 +8132,7 @@
         </is>
       </c>
       <c r="E84" t="n">
-        <v>0.26</v>
+        <v>0.287</v>
       </c>
       <c r="F84" t="inlineStr"/>
     </row>
@@ -8158,7 +8158,7 @@
         </is>
       </c>
       <c r="E85" t="n">
-        <v>0.265</v>
+        <v>0.224</v>
       </c>
       <c r="F85" t="inlineStr"/>
     </row>
@@ -8184,7 +8184,7 @@
         </is>
       </c>
       <c r="E86" t="n">
-        <v>0.306</v>
+        <v>0.322</v>
       </c>
       <c r="F86" t="inlineStr"/>
     </row>
@@ -8210,7 +8210,7 @@
         </is>
       </c>
       <c r="E87" t="n">
-        <v>0.328</v>
+        <v>0.226</v>
       </c>
       <c r="F87" t="inlineStr"/>
     </row>
@@ -8236,7 +8236,7 @@
         </is>
       </c>
       <c r="E88" t="n">
-        <v>0.468</v>
+        <v>0.245</v>
       </c>
       <c r="F88" t="inlineStr"/>
     </row>
@@ -8262,7 +8262,7 @@
         </is>
       </c>
       <c r="E89" t="n">
-        <v>0.27</v>
+        <v>0.366</v>
       </c>
       <c r="F89" t="inlineStr"/>
     </row>
@@ -8288,7 +8288,7 @@
         </is>
       </c>
       <c r="E90" t="n">
-        <v>0.241</v>
+        <v>0.323</v>
       </c>
       <c r="F90" t="inlineStr"/>
     </row>
@@ -8314,7 +8314,7 @@
         </is>
       </c>
       <c r="E91" t="n">
-        <v>0.306</v>
+        <v>0.223</v>
       </c>
       <c r="F91" t="inlineStr"/>
     </row>
@@ -8340,7 +8340,7 @@
         </is>
       </c>
       <c r="E92" t="n">
-        <v>0.336</v>
+        <v>0.306</v>
       </c>
       <c r="F92" t="inlineStr"/>
     </row>
@@ -8366,7 +8366,7 @@
         </is>
       </c>
       <c r="E93" t="n">
-        <v>0.235</v>
+        <v>0.298</v>
       </c>
       <c r="F93" t="inlineStr"/>
     </row>
@@ -8392,7 +8392,7 @@
         </is>
       </c>
       <c r="E94" t="n">
-        <v>0.419</v>
+        <v>1.906</v>
       </c>
       <c r="F94" t="inlineStr"/>
     </row>
@@ -8418,7 +8418,7 @@
         </is>
       </c>
       <c r="E95" t="n">
-        <v>0.574</v>
+        <v>1.084</v>
       </c>
       <c r="F95" t="inlineStr"/>
     </row>
@@ -8444,7 +8444,7 @@
         </is>
       </c>
       <c r="E96" t="n">
-        <v>0.29</v>
+        <v>0.277</v>
       </c>
       <c r="F96" t="inlineStr"/>
     </row>
@@ -8470,7 +8470,7 @@
         </is>
       </c>
       <c r="E97" t="n">
-        <v>0.271</v>
+        <v>0.421</v>
       </c>
       <c r="F97" t="inlineStr"/>
     </row>
@@ -8496,7 +8496,7 @@
         </is>
       </c>
       <c r="E98" t="n">
-        <v>0.306</v>
+        <v>0.347</v>
       </c>
       <c r="F98" t="inlineStr"/>
     </row>
@@ -8522,7 +8522,7 @@
         </is>
       </c>
       <c r="E99" t="n">
-        <v>0.363</v>
+        <v>0.319</v>
       </c>
       <c r="F99" t="inlineStr"/>
     </row>
@@ -8548,7 +8548,7 @@
         </is>
       </c>
       <c r="E100" t="n">
-        <v>0.358</v>
+        <v>0.338</v>
       </c>
       <c r="F100" t="inlineStr"/>
     </row>
@@ -8574,7 +8574,7 @@
         </is>
       </c>
       <c r="E101" t="n">
-        <v>0.263</v>
+        <v>0.38</v>
       </c>
       <c r="F101" t="inlineStr"/>
     </row>
@@ -13938,7 +13938,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>2.189</v>
+        <v>4.234</v>
       </c>
       <c r="F2" t="inlineStr"/>
     </row>
@@ -13964,7 +13964,7 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>0.321</v>
+        <v>3.317</v>
       </c>
       <c r="F3" t="inlineStr"/>
     </row>
@@ -13990,7 +13990,7 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>0.631</v>
+        <v>3.336</v>
       </c>
       <c r="F4" t="inlineStr"/>
     </row>
@@ -14016,7 +14016,7 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>0.382</v>
+        <v>3.285</v>
       </c>
       <c r="F5" t="inlineStr"/>
     </row>
@@ -14042,7 +14042,7 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>0.267</v>
+        <v>3.343</v>
       </c>
       <c r="F6" t="inlineStr"/>
     </row>
@@ -14068,7 +14068,7 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>0.346</v>
+        <v>3.224</v>
       </c>
       <c r="F7" t="inlineStr"/>
     </row>
@@ -14094,7 +14094,7 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>0.447</v>
+        <v>3.267</v>
       </c>
       <c r="F8" t="inlineStr"/>
     </row>
@@ -14120,7 +14120,7 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>0.297</v>
+        <v>1.597</v>
       </c>
       <c r="F9" t="inlineStr"/>
     </row>
@@ -14146,7 +14146,7 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>0.331</v>
+        <v>0.891</v>
       </c>
       <c r="F10" t="inlineStr"/>
     </row>
@@ -14172,7 +14172,7 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>0.355</v>
+        <v>0.984</v>
       </c>
       <c r="F11" t="inlineStr"/>
     </row>
@@ -14198,7 +14198,7 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>0.248</v>
+        <v>0.224</v>
       </c>
       <c r="F12" t="inlineStr"/>
     </row>
@@ -14224,7 +14224,7 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>0.349</v>
+        <v>0.351</v>
       </c>
       <c r="F13" t="inlineStr"/>
     </row>
@@ -14250,7 +14250,7 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>0.235</v>
+        <v>0.223</v>
       </c>
       <c r="F14" t="inlineStr"/>
     </row>
@@ -14276,7 +14276,7 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>0.283</v>
+        <v>0.254</v>
       </c>
       <c r="F15" t="inlineStr"/>
     </row>
@@ -14302,7 +14302,7 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>0.343</v>
+        <v>0.281</v>
       </c>
       <c r="F16" t="inlineStr"/>
     </row>
@@ -14328,7 +14328,7 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>0.369</v>
+        <v>0.219</v>
       </c>
       <c r="F17" t="inlineStr"/>
     </row>
@@ -14354,7 +14354,7 @@
         </is>
       </c>
       <c r="E18" t="n">
-        <v>0.355</v>
+        <v>0.232</v>
       </c>
       <c r="F18" t="inlineStr"/>
     </row>
@@ -14380,7 +14380,7 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>0.386</v>
+        <v>0.285</v>
       </c>
       <c r="F19" t="inlineStr"/>
     </row>
@@ -14406,7 +14406,7 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>0.427</v>
+        <v>0.217</v>
       </c>
       <c r="F20" t="inlineStr"/>
     </row>
@@ -14432,7 +14432,7 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>0.28</v>
+        <v>0.242</v>
       </c>
       <c r="F21" t="inlineStr"/>
     </row>
@@ -14458,7 +14458,7 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>0.58</v>
+        <v>0.284</v>
       </c>
       <c r="F22" t="inlineStr"/>
     </row>
@@ -14484,7 +14484,7 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>0.307</v>
+        <v>0.226</v>
       </c>
       <c r="F23" t="inlineStr"/>
     </row>
@@ -14510,7 +14510,7 @@
         </is>
       </c>
       <c r="E24" t="n">
-        <v>0.311</v>
+        <v>0.238</v>
       </c>
       <c r="F24" t="inlineStr"/>
     </row>
@@ -14536,7 +14536,7 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>0.296</v>
+        <v>0.223</v>
       </c>
       <c r="F25" t="inlineStr"/>
     </row>
@@ -14562,7 +14562,7 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>0.246</v>
+        <v>0.235</v>
       </c>
       <c r="F26" t="inlineStr"/>
     </row>
@@ -14588,7 +14588,7 @@
         </is>
       </c>
       <c r="E27" t="n">
-        <v>0.54</v>
+        <v>0.225</v>
       </c>
       <c r="F27" t="inlineStr"/>
     </row>
@@ -14614,7 +14614,7 @@
         </is>
       </c>
       <c r="E28" t="n">
-        <v>0.346</v>
+        <v>0.249</v>
       </c>
       <c r="F28" t="inlineStr"/>
     </row>
@@ -14640,7 +14640,7 @@
         </is>
       </c>
       <c r="E29" t="n">
-        <v>0.548</v>
+        <v>0.296</v>
       </c>
       <c r="F29" t="inlineStr"/>
     </row>
@@ -14666,7 +14666,7 @@
         </is>
       </c>
       <c r="E30" t="n">
-        <v>0.967</v>
+        <v>0.222</v>
       </c>
       <c r="F30" t="inlineStr"/>
     </row>
@@ -14692,7 +14692,7 @@
         </is>
       </c>
       <c r="E31" t="n">
-        <v>0.281</v>
+        <v>0.223</v>
       </c>
       <c r="F31" t="inlineStr"/>
     </row>
@@ -14718,7 +14718,7 @@
         </is>
       </c>
       <c r="E32" t="n">
-        <v>0.403</v>
+        <v>0.375</v>
       </c>
       <c r="F32" t="inlineStr"/>
     </row>
@@ -14744,7 +14744,7 @@
         </is>
       </c>
       <c r="E33" t="n">
-        <v>0.294</v>
+        <v>0.246</v>
       </c>
       <c r="F33" t="inlineStr"/>
     </row>
@@ -14770,7 +14770,7 @@
         </is>
       </c>
       <c r="E34" t="n">
-        <v>0.249</v>
+        <v>0.252</v>
       </c>
       <c r="F34" t="inlineStr"/>
     </row>
@@ -14796,7 +14796,7 @@
         </is>
       </c>
       <c r="E35" t="n">
-        <v>0.338</v>
+        <v>0.255</v>
       </c>
       <c r="F35" t="inlineStr"/>
     </row>
@@ -14822,7 +14822,7 @@
         </is>
       </c>
       <c r="E36" t="n">
-        <v>0.238</v>
+        <v>0.302</v>
       </c>
       <c r="F36" t="inlineStr"/>
     </row>
@@ -14848,7 +14848,7 @@
         </is>
       </c>
       <c r="E37" t="n">
-        <v>0.305</v>
+        <v>0.246</v>
       </c>
       <c r="F37" t="inlineStr"/>
     </row>
@@ -14874,7 +14874,7 @@
         </is>
       </c>
       <c r="E38" t="n">
-        <v>0.725</v>
+        <v>0.231</v>
       </c>
       <c r="F38" t="inlineStr"/>
     </row>
@@ -14900,7 +14900,7 @@
         </is>
       </c>
       <c r="E39" t="n">
-        <v>0.319</v>
+        <v>0.22</v>
       </c>
       <c r="F39" t="inlineStr"/>
     </row>
@@ -14926,7 +14926,7 @@
         </is>
       </c>
       <c r="E40" t="n">
-        <v>0.426</v>
+        <v>0.407</v>
       </c>
       <c r="F40" t="inlineStr"/>
     </row>
@@ -14952,7 +14952,7 @@
         </is>
       </c>
       <c r="E41" t="n">
-        <v>0.252</v>
+        <v>0.222</v>
       </c>
       <c r="F41" t="inlineStr"/>
     </row>
@@ -14978,7 +14978,7 @@
         </is>
       </c>
       <c r="E42" t="n">
-        <v>0.543</v>
+        <v>0.832</v>
       </c>
       <c r="F42" t="inlineStr"/>
     </row>
@@ -15030,7 +15030,7 @@
         </is>
       </c>
       <c r="E44" t="n">
-        <v>0.326</v>
+        <v>0.443</v>
       </c>
       <c r="F44" t="inlineStr"/>
     </row>
@@ -15056,7 +15056,7 @@
         </is>
       </c>
       <c r="E45" t="n">
-        <v>0.248</v>
+        <v>0.29</v>
       </c>
       <c r="F45" t="inlineStr"/>
     </row>
@@ -15082,7 +15082,7 @@
         </is>
       </c>
       <c r="E46" t="n">
-        <v>0.239</v>
+        <v>0.227</v>
       </c>
       <c r="F46" t="inlineStr"/>
     </row>
@@ -15108,7 +15108,7 @@
         </is>
       </c>
       <c r="E47" t="n">
-        <v>0.898</v>
+        <v>0.219</v>
       </c>
       <c r="F47" t="inlineStr"/>
     </row>
@@ -15134,7 +15134,7 @@
         </is>
       </c>
       <c r="E48" t="n">
-        <v>0.246</v>
+        <v>0.758</v>
       </c>
       <c r="F48" t="inlineStr"/>
     </row>
@@ -15160,7 +15160,7 @@
         </is>
       </c>
       <c r="E49" t="n">
-        <v>0.374</v>
+        <v>0.261</v>
       </c>
       <c r="F49" t="inlineStr"/>
     </row>
@@ -15186,7 +15186,7 @@
         </is>
       </c>
       <c r="E50" t="n">
-        <v>0.303</v>
+        <v>0.219</v>
       </c>
       <c r="F50" t="inlineStr"/>
     </row>
@@ -15212,7 +15212,7 @@
         </is>
       </c>
       <c r="E51" t="n">
-        <v>0.239</v>
+        <v>0.22</v>
       </c>
       <c r="F51" t="inlineStr"/>
     </row>
@@ -15238,7 +15238,7 @@
         </is>
       </c>
       <c r="E52" t="n">
-        <v>0.263</v>
+        <v>0.22</v>
       </c>
       <c r="F52" t="inlineStr"/>
     </row>
@@ -15264,7 +15264,7 @@
         </is>
       </c>
       <c r="E53" t="n">
-        <v>0.29</v>
+        <v>0.252</v>
       </c>
       <c r="F53" t="inlineStr"/>
     </row>
@@ -15290,7 +15290,7 @@
         </is>
       </c>
       <c r="E54" t="n">
-        <v>0.247</v>
+        <v>0.262</v>
       </c>
       <c r="F54" t="inlineStr"/>
     </row>
@@ -15316,7 +15316,7 @@
         </is>
       </c>
       <c r="E55" t="n">
-        <v>0.294</v>
+        <v>2.016</v>
       </c>
       <c r="F55" t="inlineStr"/>
     </row>
@@ -15342,7 +15342,7 @@
         </is>
       </c>
       <c r="E56" t="n">
-        <v>0.246</v>
+        <v>4.025</v>
       </c>
       <c r="F56" t="inlineStr"/>
     </row>
@@ -15368,7 +15368,7 @@
         </is>
       </c>
       <c r="E57" t="n">
-        <v>0.263</v>
+        <v>2.127</v>
       </c>
       <c r="F57" t="inlineStr"/>
     </row>
@@ -15394,7 +15394,7 @@
         </is>
       </c>
       <c r="E58" t="n">
-        <v>0.407</v>
+        <v>1.194</v>
       </c>
       <c r="F58" t="inlineStr"/>
     </row>
@@ -15420,7 +15420,7 @@
         </is>
       </c>
       <c r="E59" t="n">
-        <v>0.245</v>
+        <v>0.575</v>
       </c>
       <c r="F59" t="inlineStr"/>
     </row>
@@ -15446,7 +15446,7 @@
         </is>
       </c>
       <c r="E60" t="n">
-        <v>0.266</v>
+        <v>0.286</v>
       </c>
       <c r="F60" t="inlineStr"/>
     </row>
@@ -15472,7 +15472,7 @@
         </is>
       </c>
       <c r="E61" t="n">
-        <v>0.62</v>
+        <v>0.283</v>
       </c>
       <c r="F61" t="inlineStr"/>
     </row>
@@ -15498,7 +15498,7 @@
         </is>
       </c>
       <c r="E62" t="n">
-        <v>0.293</v>
+        <v>0.337</v>
       </c>
       <c r="F62" t="inlineStr"/>
     </row>
@@ -15524,7 +15524,7 @@
         </is>
       </c>
       <c r="E63" t="n">
-        <v>0.871</v>
+        <v>0.283</v>
       </c>
       <c r="F63" t="inlineStr"/>
     </row>
@@ -15550,7 +15550,7 @@
         </is>
       </c>
       <c r="E64" t="n">
-        <v>0.509</v>
+        <v>0.241</v>
       </c>
       <c r="F64" t="inlineStr"/>
     </row>
@@ -15576,7 +15576,7 @@
         </is>
       </c>
       <c r="E65" t="n">
-        <v>0.245</v>
+        <v>0.414</v>
       </c>
       <c r="F65" t="inlineStr"/>
     </row>
@@ -15602,7 +15602,7 @@
         </is>
       </c>
       <c r="E66" t="n">
-        <v>0.315</v>
+        <v>0.477</v>
       </c>
       <c r="F66" t="inlineStr"/>
     </row>
@@ -15628,7 +15628,7 @@
         </is>
       </c>
       <c r="E67" t="n">
-        <v>0.337</v>
+        <v>0.24</v>
       </c>
       <c r="F67" t="inlineStr"/>
     </row>
@@ -15654,7 +15654,7 @@
         </is>
       </c>
       <c r="E68" t="n">
-        <v>0.334</v>
+        <v>0.297</v>
       </c>
       <c r="F68" t="inlineStr"/>
     </row>
@@ -15680,7 +15680,7 @@
         </is>
       </c>
       <c r="E69" t="n">
-        <v>0.496</v>
+        <v>0.308</v>
       </c>
       <c r="F69" t="inlineStr"/>
     </row>
@@ -15706,7 +15706,7 @@
         </is>
       </c>
       <c r="E70" t="n">
-        <v>0.255</v>
+        <v>0.236</v>
       </c>
       <c r="F70" t="inlineStr"/>
     </row>
@@ -15732,7 +15732,7 @@
         </is>
       </c>
       <c r="E71" t="n">
-        <v>0.389</v>
+        <v>0.24</v>
       </c>
       <c r="F71" t="inlineStr"/>
     </row>
@@ -15758,7 +15758,7 @@
         </is>
       </c>
       <c r="E72" t="n">
-        <v>0.224</v>
+        <v>0.269</v>
       </c>
       <c r="F72" t="inlineStr"/>
     </row>
@@ -15784,7 +15784,7 @@
         </is>
       </c>
       <c r="E73" t="n">
-        <v>0.232</v>
+        <v>0.274</v>
       </c>
       <c r="F73" t="inlineStr"/>
     </row>
@@ -15810,7 +15810,7 @@
         </is>
       </c>
       <c r="E74" t="n">
-        <v>0.34</v>
+        <v>0.24</v>
       </c>
       <c r="F74" t="inlineStr"/>
     </row>
@@ -15836,7 +15836,7 @@
         </is>
       </c>
       <c r="E75" t="n">
-        <v>0.276</v>
+        <v>0.641</v>
       </c>
       <c r="F75" t="inlineStr"/>
     </row>
@@ -15862,7 +15862,7 @@
         </is>
       </c>
       <c r="E76" t="n">
-        <v>0.703</v>
+        <v>0.611</v>
       </c>
       <c r="F76" t="inlineStr"/>
     </row>
@@ -15888,7 +15888,7 @@
         </is>
       </c>
       <c r="E77" t="n">
-        <v>0.37</v>
+        <v>0.25</v>
       </c>
       <c r="F77" t="inlineStr"/>
     </row>
@@ -15914,7 +15914,7 @@
         </is>
       </c>
       <c r="E78" t="n">
-        <v>0.259</v>
+        <v>0.342</v>
       </c>
       <c r="F78" t="inlineStr"/>
     </row>
@@ -15940,7 +15940,7 @@
         </is>
       </c>
       <c r="E79" t="n">
-        <v>0.242</v>
+        <v>0.771</v>
       </c>
       <c r="F79" t="inlineStr"/>
     </row>
@@ -15966,7 +15966,7 @@
         </is>
       </c>
       <c r="E80" t="n">
-        <v>0.251</v>
+        <v>0.599</v>
       </c>
       <c r="F80" t="inlineStr"/>
     </row>
@@ -15992,7 +15992,7 @@
         </is>
       </c>
       <c r="E81" t="n">
-        <v>0.281</v>
+        <v>0.488</v>
       </c>
       <c r="F81" t="inlineStr"/>
     </row>
@@ -16018,7 +16018,7 @@
         </is>
       </c>
       <c r="E82" t="n">
-        <v>0.31</v>
+        <v>0.244</v>
       </c>
       <c r="F82" t="inlineStr"/>
     </row>
@@ -16044,7 +16044,7 @@
         </is>
       </c>
       <c r="E83" t="n">
-        <v>0.26</v>
+        <v>0.575</v>
       </c>
       <c r="F83" t="inlineStr"/>
     </row>
@@ -16070,7 +16070,7 @@
         </is>
       </c>
       <c r="E84" t="n">
-        <v>0.26</v>
+        <v>0.287</v>
       </c>
       <c r="F84" t="inlineStr"/>
     </row>
@@ -16096,7 +16096,7 @@
         </is>
       </c>
       <c r="E85" t="n">
-        <v>0.265</v>
+        <v>0.224</v>
       </c>
       <c r="F85" t="inlineStr"/>
     </row>
@@ -16122,7 +16122,7 @@
         </is>
       </c>
       <c r="E86" t="n">
-        <v>0.306</v>
+        <v>0.322</v>
       </c>
       <c r="F86" t="inlineStr"/>
     </row>
@@ -16148,7 +16148,7 @@
         </is>
       </c>
       <c r="E87" t="n">
-        <v>0.328</v>
+        <v>0.226</v>
       </c>
       <c r="F87" t="inlineStr"/>
     </row>
@@ -16174,7 +16174,7 @@
         </is>
       </c>
       <c r="E88" t="n">
-        <v>0.468</v>
+        <v>0.245</v>
       </c>
       <c r="F88" t="inlineStr"/>
     </row>
@@ -16200,7 +16200,7 @@
         </is>
       </c>
       <c r="E89" t="n">
-        <v>0.27</v>
+        <v>0.366</v>
       </c>
       <c r="F89" t="inlineStr"/>
     </row>
@@ -16226,7 +16226,7 @@
         </is>
       </c>
       <c r="E90" t="n">
-        <v>0.241</v>
+        <v>0.323</v>
       </c>
       <c r="F90" t="inlineStr"/>
     </row>
@@ -16252,7 +16252,7 @@
         </is>
       </c>
       <c r="E91" t="n">
-        <v>0.306</v>
+        <v>0.223</v>
       </c>
       <c r="F91" t="inlineStr"/>
     </row>
@@ -16278,7 +16278,7 @@
         </is>
       </c>
       <c r="E92" t="n">
-        <v>0.336</v>
+        <v>0.306</v>
       </c>
       <c r="F92" t="inlineStr"/>
     </row>
@@ -16304,7 +16304,7 @@
         </is>
       </c>
       <c r="E93" t="n">
-        <v>0.235</v>
+        <v>0.298</v>
       </c>
       <c r="F93" t="inlineStr"/>
     </row>
@@ -16330,7 +16330,7 @@
         </is>
       </c>
       <c r="E94" t="n">
-        <v>0.419</v>
+        <v>1.906</v>
       </c>
       <c r="F94" t="inlineStr"/>
     </row>
@@ -16356,7 +16356,7 @@
         </is>
       </c>
       <c r="E95" t="n">
-        <v>0.574</v>
+        <v>1.084</v>
       </c>
       <c r="F95" t="inlineStr"/>
     </row>
@@ -16382,7 +16382,7 @@
         </is>
       </c>
       <c r="E96" t="n">
-        <v>0.29</v>
+        <v>0.277</v>
       </c>
       <c r="F96" t="inlineStr"/>
     </row>
@@ -16408,7 +16408,7 @@
         </is>
       </c>
       <c r="E97" t="n">
-        <v>0.271</v>
+        <v>0.421</v>
       </c>
       <c r="F97" t="inlineStr"/>
     </row>
@@ -16434,7 +16434,7 @@
         </is>
       </c>
       <c r="E98" t="n">
-        <v>0.306</v>
+        <v>0.347</v>
       </c>
       <c r="F98" t="inlineStr"/>
     </row>
@@ -16460,7 +16460,7 @@
         </is>
       </c>
       <c r="E99" t="n">
-        <v>0.363</v>
+        <v>0.319</v>
       </c>
       <c r="F99" t="inlineStr"/>
     </row>
@@ -16486,7 +16486,7 @@
         </is>
       </c>
       <c r="E100" t="n">
-        <v>0.358</v>
+        <v>0.338</v>
       </c>
       <c r="F100" t="inlineStr"/>
     </row>
@@ -16512,7 +16512,7 @@
         </is>
       </c>
       <c r="E101" t="n">
-        <v>0.263</v>
+        <v>0.38</v>
       </c>
       <c r="F101" t="inlineStr"/>
     </row>

</xml_diff>